<commit_message>
Updated with latest annotation labels Sep22
</commit_message>
<xml_diff>
--- a/annotation/Species_list.xlsx
+++ b/annotation/Species_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25128"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hillna\OneDrive - University of Tasmania\UTAS_work\Projects\Benthic Diversity ARC\Analysis\ARC_Data\annotation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universitytasmania-my.sharepoint.com/personal/nicole_hill_utas_edu_au/Documents/UTAS_work/Projects/Benthic Diversity ARC/Analysis/ARC_Data/annotation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B109CE25-02AB-4EA7-88FB-9C74B744BE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{B109CE25-02AB-4EA7-88FB-9C74B744BE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D782C1A-F1D0-4AA8-8665-F7B533DA7E3F}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="21930" windowHeight="13830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER_prevalence" sheetId="1" r:id="rId1"/>
@@ -1198,17 +1198,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G148"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="54" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="28.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="5" max="6" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1231,7 +1231,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>0.81499999999999995</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>0.76200000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1275,7 +1275,7 @@
         <v>0.51100000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>0.48599999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>0.33200000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>0.318</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -1333,7 +1333,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>0.27700000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -1355,7 +1355,7 @@
         <v>0.26700000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1366,7 +1366,7 @@
         <v>0.26200000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>0.22800000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>18</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>0.224</v>
       </c>
     </row>
-    <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>20</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>0.192</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>0.192</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>0.17299999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>0.17199999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>0.158</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>0.156</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>31</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>32</v>
       </c>
@@ -1554,7 +1554,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>0.125</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>0.107</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>38</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>0.106</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>39</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>40</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>41</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>42</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>43</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>45</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>46</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>47</v>
       </c>
@@ -1734,7 +1734,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="45" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>48</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>49</v>
       </c>
@@ -1762,7 +1762,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>50</v>
       </c>
@@ -1773,7 +1773,7 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>51</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>52</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>8.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>53</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>8.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>54</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>7.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>55</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>7.8E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>56</v>
       </c>
@@ -1845,7 +1845,7 @@
         <v>7.0999999999999994E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>6.9000000000000006E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>58</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>59</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>60</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>6.3E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>61</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>6.2E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>62</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>63</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>5.8000000000000003E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>64</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>65</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>66</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>67</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>68</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>69</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>70</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="68" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>71</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>72</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>73</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>74</v>
       </c>
@@ -2058,7 +2058,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>75</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>76</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>3.9E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>77</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>78</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -2116,7 +2116,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>80</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>81</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>82</v>
       </c>
@@ -2152,7 +2152,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -2163,7 +2163,7 @@
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>84</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>85</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>86</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>87</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="85" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>88</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="86" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>89</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="87" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>90</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>91</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>92</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>2.3E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>93</v>
       </c>
@@ -2285,7 +2285,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>94</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>95</v>
       </c>
@@ -2307,7 +2307,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>96</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="94" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>97</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="95" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>98</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>99</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>100</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>101</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>102</v>
       </c>
@@ -2402,7 +2402,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>103</v>
       </c>
@@ -2416,7 +2416,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>104</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>105</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="103" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
         <v>106</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="104" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
         <v>107</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>108</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>109</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>110</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>111</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
         <v>112</v>
       </c>
@@ -2542,7 +2542,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>113</v>
       </c>
@@ -2556,7 +2556,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>114</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>115</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>116</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="114" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="7" t="s">
         <v>117</v>
       </c>
@@ -2612,7 +2612,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>118</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="116" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
         <v>119</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>120</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="118" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
         <v>121</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="119" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
         <v>122</v>
       </c>
@@ -2685,7 +2685,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="120" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
         <v>123</v>
       </c>
@@ -2699,7 +2699,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>124</v>
       </c>
@@ -2716,7 +2716,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>125</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="123" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
         <v>126</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>127</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>128</v>
       </c>
@@ -2781,7 +2781,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="126" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="8" t="s">
         <v>129</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="127" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>130</v>
       </c>
@@ -2812,7 +2812,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="128" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
         <v>131</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="129" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="6" t="s">
         <v>132</v>
       </c>
@@ -2840,7 +2840,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>133</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="131" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
         <v>134</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="132" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>135</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="133" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
         <v>136</v>
       </c>
@@ -2899,7 +2899,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="134" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
         <v>137</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="135" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>138</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="136" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
         <v>139</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="137" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
         <v>140</v>
       </c>
@@ -2958,7 +2958,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="138" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
         <v>141</v>
       </c>
@@ -2972,7 +2972,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>142</v>
       </c>
@@ -2989,7 +2989,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>143</v>
       </c>
@@ -3006,7 +3006,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="141" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
         <v>144</v>
       </c>
@@ -3020,7 +3020,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="142" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
         <v>145</v>
       </c>
@@ -3034,7 +3034,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="143" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
         <v>146</v>
       </c>
@@ -3048,7 +3048,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="144" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="5" t="s">
         <v>147</v>
       </c>
@@ -3062,7 +3062,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="145" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="5" t="s">
         <v>148</v>
       </c>
@@ -3076,7 +3076,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="146" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
         <v>149</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="147" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>150</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="148" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
         <v>151</v>
       </c>
@@ -3127,9 +3127,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B148"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>152</v>
       </c>
@@ -3137,7 +3137,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>56.216999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>20.123999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3161,7 +3161,7 @@
         <v>3.8090000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>3.0350000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3177,7 +3177,7 @@
         <v>2.4790000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>1.982</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -3193,7 +3193,7 @@
         <v>1.1259999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -3201,7 +3201,7 @@
         <v>1.0589999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -3209,7 +3209,7 @@
         <v>0.77400000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -3217,7 +3217,7 @@
         <v>0.65600000000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>0.54800000000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>0.44800000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>0.436</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>0.39900000000000002</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>0.35199999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>0.35199999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>0.33100000000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>0.32800000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -3297,7 +3297,7 @@
         <v>0.32800000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -3305,7 +3305,7 @@
         <v>0.27700000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -3313,7 +3313,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -3321,7 +3321,7 @@
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>102</v>
       </c>
@@ -3337,7 +3337,7 @@
         <v>0.14499999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -3345,7 +3345,7 @@
         <v>0.129</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>99</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>37</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>0.126</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -3369,7 +3369,7 @@
         <v>0.121</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>18</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>0.114</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>0.10100000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>65</v>
       </c>
@@ -3417,7 +3417,7 @@
         <v>9.8000000000000004E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>34</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>31</v>
       </c>
@@ -3433,7 +3433,7 @@
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>22</v>
       </c>
@@ -3441,7 +3441,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>36</v>
       </c>
@@ -3449,7 +3449,7 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>38</v>
       </c>
@@ -3457,7 +3457,7 @@
         <v>8.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>25</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>7.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>79</v>
       </c>
@@ -3481,7 +3481,7 @@
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>42</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>6.6000000000000003E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>53</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>40</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>6.3E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>61</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>6.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>50</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>5.8000000000000003E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>86</v>
       </c>
@@ -3529,7 +3529,7 @@
         <v>5.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>27</v>
       </c>
@@ -3537,7 +3537,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>49</v>
       </c>
@@ -3545,7 +3545,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>60</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>4.7E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -3561,7 +3561,7 @@
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>72</v>
       </c>
@@ -3569,7 +3569,7 @@
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>46</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>104</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>41</v>
       </c>
@@ -3593,7 +3593,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>55</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>83</v>
       </c>
@@ -3609,7 +3609,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>74</v>
       </c>
@@ -3617,7 +3617,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>77</v>
       </c>
@@ -3625,7 +3625,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>82</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>52</v>
       </c>
@@ -3641,7 +3641,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>48</v>
       </c>
@@ -3649,7 +3649,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>47</v>
       </c>
@@ -3657,7 +3657,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>96</v>
       </c>
@@ -3665,7 +3665,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>43</v>
       </c>
@@ -3673,7 +3673,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>58</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>76</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>93</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>59</v>
       </c>
@@ -3705,7 +3705,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>63</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>62</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>97</v>
       </c>
@@ -3729,7 +3729,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>64</v>
       </c>
@@ -3737,7 +3737,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>137</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>75</v>
       </c>
@@ -3753,7 +3753,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>73</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>2.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>56</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>68</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>100</v>
       </c>
@@ -3785,7 +3785,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>115</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>66</v>
       </c>
@@ -3801,7 +3801,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>90</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>136</v>
       </c>
@@ -3817,7 +3817,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>78</v>
       </c>
@@ -3825,7 +3825,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>80</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>81</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>69</v>
       </c>
@@ -3849,7 +3849,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>70</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>108</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>143</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>84</v>
       </c>
@@ -3881,7 +3881,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>71</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>94</v>
       </c>
@@ -3897,7 +3897,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>117</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>88</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>87</v>
       </c>
@@ -3921,7 +3921,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>85</v>
       </c>
@@ -3929,7 +3929,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>101</v>
       </c>
@@ -3937,7 +3937,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>118</v>
       </c>
@@ -3945,7 +3945,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>113</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>106</v>
       </c>
@@ -3961,7 +3961,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>95</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>92</v>
       </c>
@@ -3977,7 +3977,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>129</v>
       </c>
@@ -3985,7 +3985,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>124</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>125</v>
       </c>
@@ -4001,7 +4001,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>103</v>
       </c>
@@ -4009,7 +4009,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>147</v>
       </c>
@@ -4017,7 +4017,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>89</v>
       </c>
@@ -4025,7 +4025,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>91</v>
       </c>
@@ -4033,7 +4033,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>98</v>
       </c>
@@ -4041,7 +4041,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>111</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>109</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>127</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>110</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>114</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>105</v>
       </c>
@@ -4089,7 +4089,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>107</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>120</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>126</v>
       </c>
@@ -4113,7 +4113,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>116</v>
       </c>
@@ -4121,7 +4121,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>112</v>
       </c>
@@ -4129,7 +4129,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>133</v>
       </c>
@@ -4137,7 +4137,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>119</v>
       </c>
@@ -4145,7 +4145,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>128</v>
       </c>
@@ -4153,7 +4153,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>138</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>123</v>
       </c>
@@ -4169,7 +4169,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>122</v>
       </c>
@@ -4177,7 +4177,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>134</v>
       </c>
@@ -4185,7 +4185,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>121</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>132</v>
       </c>
@@ -4201,7 +4201,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>130</v>
       </c>
@@ -4209,7 +4209,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>141</v>
       </c>
@@ -4217,7 +4217,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>131</v>
       </c>
@@ -4225,7 +4225,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>146</v>
       </c>
@@ -4233,7 +4233,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>135</v>
       </c>
@@ -4241,7 +4241,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>139</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>140</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>142</v>
       </c>
@@ -4265,7 +4265,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>144</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>145</v>
       </c>
@@ -4281,7 +4281,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>148</v>
       </c>
@@ -4289,7 +4289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>149</v>
       </c>
@@ -4297,7 +4297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>150</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>151</v>
       </c>
@@ -4321,17 +4321,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G89"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4354,7 +4354,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
@@ -4365,7 +4365,7 @@
         <v>0.94099999999999995</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>155</v>
       </c>
@@ -4382,7 +4382,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>156</v>
       </c>
@@ -4393,7 +4393,7 @@
         <v>0.71399999999999997</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>157</v>
       </c>
@@ -4404,7 +4404,7 @@
         <v>0.621</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>158</v>
       </c>
@@ -4415,7 +4415,7 @@
         <v>0.53600000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4426,7 +4426,7 @@
         <v>0.52100000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>159</v>
       </c>
@@ -4437,7 +4437,7 @@
         <v>0.503</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>160</v>
       </c>
@@ -4448,7 +4448,7 @@
         <v>0.47799999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>161</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>0.435</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>162</v>
       </c>
@@ -4470,7 +4470,7 @@
         <v>0.38500000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>163</v>
       </c>
@@ -4481,7 +4481,7 @@
         <v>0.29499999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>164</v>
       </c>
@@ -4492,7 +4492,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>165</v>
       </c>
@@ -4503,7 +4503,7 @@
         <v>0.26700000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>166</v>
       </c>
@@ -4514,7 +4514,7 @@
         <v>0.26500000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>167</v>
       </c>
@@ -4525,7 +4525,7 @@
         <v>0.23100000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>168</v>
       </c>
@@ -4536,7 +4536,7 @@
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>169</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>0.20899999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>170</v>
       </c>
@@ -4558,7 +4558,7 @@
         <v>0.20300000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>171</v>
       </c>
@@ -4569,7 +4569,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>172</v>
       </c>
@@ -4580,7 +4580,7 @@
         <v>0.186</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>173</v>
       </c>
@@ -4591,7 +4591,7 @@
         <v>0.155</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>174</v>
       </c>
@@ -4602,7 +4602,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>175</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>176</v>
       </c>
@@ -4630,7 +4630,7 @@
         <v>0.13200000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>177</v>
       </c>
@@ -4647,7 +4647,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>178</v>
       </c>
@@ -4658,7 +4658,7 @@
         <v>0.11899999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>179</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>0.109</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>180</v>
       </c>
@@ -4680,7 +4680,7 @@
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>181</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>9.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>182</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>9.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>183</v>
       </c>
@@ -4713,7 +4713,7 @@
         <v>9.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>184</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>8.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>185</v>
       </c>
@@ -4735,7 +4735,7 @@
         <v>7.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>186</v>
       </c>
@@ -4746,7 +4746,7 @@
         <v>7.5999999999999998E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>187</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>188</v>
       </c>
@@ -4774,7 +4774,7 @@
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>189</v>
       </c>
@@ -4785,7 +4785,7 @@
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>190</v>
       </c>
@@ -4796,7 +4796,7 @@
         <v>6.7000000000000004E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>191</v>
       </c>
@@ -4807,7 +4807,7 @@
         <v>6.6000000000000003E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>192</v>
       </c>
@@ -4818,7 +4818,7 @@
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>193</v>
       </c>
@@ -4829,7 +4829,7 @@
         <v>6.2E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>194</v>
       </c>
@@ -4840,7 +4840,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>195</v>
       </c>
@@ -4851,7 +4851,7 @@
         <v>5.8000000000000003E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>196</v>
       </c>
@@ -4862,7 +4862,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>197</v>
       </c>
@@ -4876,7 +4876,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>198</v>
       </c>
@@ -4887,7 +4887,7 @@
         <v>5.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>199</v>
       </c>
@@ -4898,7 +4898,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>200</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>201</v>
       </c>
@@ -4920,7 +4920,7 @@
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>202</v>
       </c>
@@ -4934,7 +4934,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>203</v>
       </c>
@@ -4945,7 +4945,7 @@
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>204</v>
       </c>
@@ -4956,7 +4956,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>205</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>206</v>
       </c>
@@ -4978,7 +4978,7 @@
         <v>3.9E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>207</v>
       </c>
@@ -4989,7 +4989,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>130</v>
       </c>
@@ -5000,7 +5000,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>208</v>
       </c>
@@ -5011,7 +5011,7 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>209</v>
       </c>
@@ -5022,7 +5022,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>210</v>
       </c>
@@ -5039,7 +5039,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>211</v>
       </c>
@@ -5050,7 +5050,7 @@
         <v>3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>212</v>
       </c>
@@ -5061,7 +5061,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>213</v>
       </c>
@@ -5072,7 +5072,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>214</v>
       </c>
@@ -5083,7 +5083,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>215</v>
       </c>
@@ -5100,7 +5100,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>216</v>
       </c>
@@ -5111,7 +5111,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>217</v>
       </c>
@@ -5122,7 +5122,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="68" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>218</v>
       </c>
@@ -5139,7 +5139,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>219</v>
       </c>
@@ -5156,7 +5156,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>220</v>
       </c>
@@ -5167,7 +5167,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>221</v>
       </c>
@@ -5178,7 +5178,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>222</v>
       </c>
@@ -5189,7 +5189,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>223</v>
       </c>
@@ -5200,7 +5200,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>224</v>
       </c>
@@ -5211,7 +5211,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>225</v>
       </c>
@@ -5222,7 +5222,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>226</v>
       </c>
@@ -5236,7 +5236,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>227</v>
       </c>
@@ -5247,7 +5247,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="78" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>228</v>
       </c>
@@ -5258,7 +5258,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>229</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>230</v>
       </c>
@@ -5280,7 +5280,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>231</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>232</v>
       </c>
@@ -5302,7 +5302,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>233</v>
       </c>
@@ -5313,7 +5313,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>234</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>235</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>236</v>
       </c>
@@ -5346,7 +5346,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>237</v>
       </c>
@@ -5357,7 +5357,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>238</v>
       </c>
@@ -5368,7 +5368,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
         <v>239</v>
       </c>
@@ -5391,12 +5391,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B89"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.7265625" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>152</v>
       </c>
@@ -5404,7 +5404,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
@@ -5412,7 +5412,7 @@
         <v>54271</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>156</v>
       </c>
@@ -5420,7 +5420,7 @@
         <v>45078</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>155</v>
       </c>
@@ -5428,7 +5428,7 @@
         <v>19844</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>161</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>7641</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>157</v>
       </c>
@@ -5444,7 +5444,7 @@
         <v>5986</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>159</v>
       </c>
@@ -5452,7 +5452,7 @@
         <v>5228</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>166</v>
       </c>
@@ -5460,7 +5460,7 @@
         <v>2577</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>165</v>
       </c>
@@ -5468,7 +5468,7 @@
         <v>2431</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>206</v>
       </c>
@@ -5476,7 +5476,7 @@
         <v>2389</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>176</v>
       </c>
@@ -5484,7 +5484,7 @@
         <v>2195</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>160</v>
       </c>
@@ -5492,7 +5492,7 @@
         <v>2128</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>162</v>
       </c>
@@ -5500,7 +5500,7 @@
         <v>1799</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>178</v>
       </c>
@@ -5508,7 +5508,7 @@
         <v>1711</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>182</v>
       </c>
@@ -5516,7 +5516,7 @@
         <v>1648</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -5524,7 +5524,7 @@
         <v>1630</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>194</v>
       </c>
@@ -5532,7 +5532,7 @@
         <v>1583</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>158</v>
       </c>
@@ -5540,7 +5540,7 @@
         <v>1577</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>183</v>
       </c>
@@ -5548,7 +5548,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>164</v>
       </c>
@@ -5556,7 +5556,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>191</v>
       </c>
@@ -5564,7 +5564,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>203</v>
       </c>
@@ -5572,7 +5572,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>168</v>
       </c>
@@ -5580,7 +5580,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>167</v>
       </c>
@@ -5588,7 +5588,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>173</v>
       </c>
@@ -5596,7 +5596,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>170</v>
       </c>
@@ -5604,7 +5604,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>216</v>
       </c>
@@ -5612,7 +5612,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>198</v>
       </c>
@@ -5620,7 +5620,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>196</v>
       </c>
@@ -5628,7 +5628,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>163</v>
       </c>
@@ -5636,7 +5636,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>172</v>
       </c>
@@ -5644,7 +5644,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>180</v>
       </c>
@@ -5652,7 +5652,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>169</v>
       </c>
@@ -5660,7 +5660,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>177</v>
       </c>
@@ -5668,7 +5668,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>238</v>
       </c>
@@ -5676,7 +5676,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>179</v>
       </c>
@@ -5684,7 +5684,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>171</v>
       </c>
@@ -5692,7 +5692,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>174</v>
       </c>
@@ -5700,7 +5700,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>185</v>
       </c>
@@ -5708,7 +5708,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>187</v>
       </c>
@@ -5716,7 +5716,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>175</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5732,7 +5732,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>184</v>
       </c>
@@ -5740,7 +5740,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>202</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>181</v>
       </c>
@@ -5756,7 +5756,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>186</v>
       </c>
@@ -5764,7 +5764,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>208</v>
       </c>
@@ -5772,7 +5772,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>211</v>
       </c>
@@ -5780,7 +5780,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>190</v>
       </c>
@@ -5788,7 +5788,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>200</v>
       </c>
@@ -5796,7 +5796,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>188</v>
       </c>
@@ -5804,7 +5804,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>130</v>
       </c>
@@ -5812,7 +5812,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>199</v>
       </c>
@@ -5820,7 +5820,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>210</v>
       </c>
@@ -5828,7 +5828,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>192</v>
       </c>
@@ -5836,7 +5836,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>193</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>195</v>
       </c>
@@ -5852,7 +5852,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>197</v>
       </c>
@@ -5860,7 +5860,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>201</v>
       </c>
@@ -5868,7 +5868,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>204</v>
       </c>
@@ -5876,7 +5876,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>205</v>
       </c>
@@ -5884,7 +5884,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>207</v>
       </c>
@@ -5892,7 +5892,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>212</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>209</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>213</v>
       </c>
@@ -5916,7 +5916,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>234</v>
       </c>
@@ -5924,7 +5924,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>220</v>
       </c>
@@ -5932,7 +5932,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>218</v>
       </c>
@@ -5940,7 +5940,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>219</v>
       </c>
@@ -5948,7 +5948,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>217</v>
       </c>
@@ -5956,7 +5956,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>214</v>
       </c>
@@ -5964,7 +5964,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>221</v>
       </c>
@@ -5972,7 +5972,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>233</v>
       </c>
@@ -5980,7 +5980,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>215</v>
       </c>
@@ -5988,7 +5988,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>223</v>
       </c>
@@ -5996,7 +5996,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>225</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>222</v>
       </c>
@@ -6012,7 +6012,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>229</v>
       </c>
@@ -6020,7 +6020,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>224</v>
       </c>
@@ -6028,7 +6028,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>226</v>
       </c>
@@ -6036,7 +6036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>227</v>
       </c>
@@ -6044,7 +6044,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>231</v>
       </c>
@@ -6052,7 +6052,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>228</v>
       </c>
@@ -6060,7 +6060,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>230</v>
       </c>
@@ -6068,7 +6068,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>232</v>
       </c>
@@ -6076,7 +6076,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>235</v>
       </c>
@@ -6084,7 +6084,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>236</v>
       </c>
@@ -6092,7 +6092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>237</v>
       </c>
@@ -6100,7 +6100,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>239</v>
       </c>

</xml_diff>